<commit_message>
changed metadat to address testcases
</commit_message>
<xml_diff>
--- a/scripts/example_input/dummy_traject/16-X_001_DP003-DP008.xlsx
+++ b/scripts/example_input/dummy_traject/16-X_001_DP003-DP008.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SAKA\sources\github\faalkansbeheer\scripts\example_input\dummy_traject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DC696DF-3584-4D2E-9556-8A4E28772C54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD04E7A2-9F87-49DC-B146-229745427DD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="scenario1" sheetId="4" r:id="rId1"/>
@@ -185,9 +185,6 @@
     <t>16-X</t>
   </si>
   <si>
-    <t>groene dijk</t>
-  </si>
-  <si>
     <t>Vervolgmechanismen</t>
   </si>
   <si>
@@ -219,6 +216,9 @@
   </si>
   <si>
     <t>Overstroming - glijvlak zonder reststerkte | geen graverij</t>
+  </si>
+  <si>
+    <t>Testcase met dierlijke graverij</t>
   </si>
 </sst>
 </file>
@@ -1118,13 +1118,13 @@
         <v>1</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F6" s="5">
         <v>500</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>40</v>
@@ -1139,10 +1139,10 @@
         <v>550</v>
       </c>
       <c r="L6" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="M6" s="6" t="s">
         <v>45</v>
-      </c>
-      <c r="M6" s="6" t="s">
-        <v>46</v>
       </c>
       <c r="N6" s="24">
         <v>7</v>
@@ -1227,10 +1227,10 @@
         <v>29</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
@@ -1250,13 +1250,13 @@
         <v>29</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
@@ -1272,13 +1272,13 @@
         <v>29</v>
       </c>
       <c r="C15" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="E15" s="8" t="s">
         <v>50</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>51</v>
       </c>
       <c r="F15" s="8"/>
       <c r="G15" s="8"/>
@@ -2243,49 +2243,55 @@
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="338e11dd-9b15-475b-8471-fcb79439c886">CBPJ-627581585-39893</_dlc_DocId>
-    <e39ed97c196f40ca8994d73dd80b64d0 xmlns="338e11dd-9b15-475b-8471-fcb79439c886">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Waterschap Rivierenland</TermName>
-          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">d1732778-9e42-4ec7-9c76-7a14861f4695</TermId>
-        </TermInfo>
-      </Terms>
-    </e39ed97c196f40ca8994d73dd80b64d0>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="edfbc03d-db26-4301-8719-99148ee26221">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="338e11dd-9b15-475b-8471-fcb79439c886">
-      <Value>2</Value>
-      <Value>1</Value>
-    </TaxCatchAll>
-    <n3c4235fe90e4626a88beeb52e343114 xmlns="338e11dd-9b15-475b-8471-fcb79439c886">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Concept</TermName>
-          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">c1e89abd-99d3-43d9-9ea5-d87afe83fe15</TermId>
-        </TermInfo>
-      </Terms>
-    </n3c4235fe90e4626a88beeb52e343114>
-    <_dlc_DocIdUrl xmlns="338e11dd-9b15-475b-8471-fcb79439c886">
-      <Url>https://wsrlnl.sharepoint.com/sites/CBPR-ydjk6ItuUw/_layouts/15/DocIdRedir.aspx?ID=CBPJ-627581585-39893</Url>
-      <Description>CBPJ-627581585-39893</Description>
-    </_dlc_DocIdUrl>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document CB" ma:contentTypeID="0x010100A075C07AB76F2344B407AD577D6B92360100C7929242D85FED4E837C6D4097594A04" ma:contentTypeVersion="17" ma:contentTypeDescription="WSRL Document CB" ma:contentTypeScope="" ma:versionID="18c34f52c90103a5ca6273d5693675c9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="338e11dd-9b15-475b-8471-fcb79439c886" xmlns:ns3="edfbc03d-db26-4301-8719-99148ee26221" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3b0dc2be265e99dcf2e366001e246f12" ns2:_="" ns3:_="">
     <xsd:import namespace="338e11dd-9b15-475b-8471-fcb79439c886"/>
@@ -2567,76 +2573,59 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="338e11dd-9b15-475b-8471-fcb79439c886">CBPJ-627581585-39893</_dlc_DocId>
+    <e39ed97c196f40ca8994d73dd80b64d0 xmlns="338e11dd-9b15-475b-8471-fcb79439c886">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Waterschap Rivierenland</TermName>
+          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">d1732778-9e42-4ec7-9c76-7a14861f4695</TermId>
+        </TermInfo>
+      </Terms>
+    </e39ed97c196f40ca8994d73dd80b64d0>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="edfbc03d-db26-4301-8719-99148ee26221">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="338e11dd-9b15-475b-8471-fcb79439c886">
+      <Value>2</Value>
+      <Value>1</Value>
+    </TaxCatchAll>
+    <n3c4235fe90e4626a88beeb52e343114 xmlns="338e11dd-9b15-475b-8471-fcb79439c886">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Concept</TermName>
+          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">c1e89abd-99d3-43d9-9ea5-d87afe83fe15</TermId>
+        </TermInfo>
+      </Terms>
+    </n3c4235fe90e4626a88beeb52e343114>
+    <_dlc_DocIdUrl xmlns="338e11dd-9b15-475b-8471-fcb79439c886">
+      <Url>https://wsrlnl.sharepoint.com/sites/CBPR-ydjk6ItuUw/_layouts/15/DocIdRedir.aspx?ID=CBPJ-627581585-39893</Url>
+      <Description>CBPJ-627581585-39893</Description>
+    </_dlc_DocIdUrl>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{263B6D11-DEF0-4FE0-9C65-6A39ECB04A89}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FB6BAA4-1CD2-494A-9433-1FC41C42B0F8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{633EBDFC-B21A-4048-98F2-0CE0F24CB488}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="338e11dd-9b15-475b-8471-fcb79439c886"/>
-    <ds:schemaRef ds:uri="edfbc03d-db26-4301-8719-99148ee26221"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC89D3C9-3D59-4FE5-907B-98550F7D511D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2655,10 +2644,21 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{633EBDFC-B21A-4048-98F2-0CE0F24CB488}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="338e11dd-9b15-475b-8471-fcb79439c886"/>
+    <ds:schemaRef ds:uri="edfbc03d-db26-4301-8719-99148ee26221"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FB6BAA4-1CD2-494A-9433-1FC41C42B0F8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{263B6D11-DEF0-4FE0-9C65-6A39ECB04A89}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
test dierlijke graverij en overslag
</commit_message>
<xml_diff>
--- a/scripts/example_input/dummy_traject/16-X_001_DP003-DP008.xlsx
+++ b/scripts/example_input/dummy_traject/16-X_001_DP003-DP008.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SAKA\sources\github\faalkansbeheer\scripts\example_input\dummy_traject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD04E7A2-9F87-49DC-B146-229745427DD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AE780E9-D8B9-4675-AA45-07E563334166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="scenario1" sheetId="4" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="52">
   <si>
     <t>Template:</t>
   </si>
@@ -185,9 +185,6 @@
     <t>16-X</t>
   </si>
   <si>
-    <t>Vervolgmechanismen</t>
-  </si>
-  <si>
     <t>DP003.-DP008.</t>
   </si>
   <si>
@@ -197,28 +194,25 @@
     <t>016-01_0145_9_BO_km0954</t>
   </si>
   <si>
-    <t>Glijvlak zonder reststerkte | graverij</t>
-  </si>
-  <si>
-    <t>Glijvak zonder reststerkte | geen graverij</t>
-  </si>
-  <si>
-    <t>Glijvlak met reststerkte | geen graverij</t>
-  </si>
-  <si>
     <t>graverij</t>
   </si>
   <si>
-    <t>Overstroming - glijvlak zonder reststerkte | graverij</t>
-  </si>
-  <si>
-    <t>Overstroming - glijvlak/vervolgmechanismen | geen graverij</t>
-  </si>
-  <si>
-    <t>Overstroming - glijvlak zonder reststerkte | geen graverij</t>
-  </si>
-  <si>
     <t>Testcase met dierlijke graverij</t>
+  </si>
+  <si>
+    <t>ja</t>
+  </si>
+  <si>
+    <t>Glijvak zonder reststerkte | geen graverij geen overslag</t>
+  </si>
+  <si>
+    <t>Glijvlak zonder reststerkte | geen graverij wel overslag</t>
+  </si>
+  <si>
+    <t>Glijvlak zonder reststerkte | graverij geen overslag</t>
+  </si>
+  <si>
+    <t>Glijvak zonder reststerkte | overslag en graverij</t>
   </si>
 </sst>
 </file>
@@ -1118,13 +1112,13 @@
         <v>1</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F6" s="5">
         <v>500</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>40</v>
@@ -1139,10 +1133,10 @@
         <v>550</v>
       </c>
       <c r="L6" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="M6" s="6" t="s">
         <v>44</v>
-      </c>
-      <c r="M6" s="6" t="s">
-        <v>45</v>
       </c>
       <c r="N6" s="24">
         <v>7</v>
@@ -1227,11 +1221,9 @@
         <v>29</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>52</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="E13" s="8"/>
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
@@ -1244,20 +1236,16 @@
         <v>2</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="C14" t="s">
         <v>29</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>51</v>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
       <c r="I14" s="8"/>
@@ -1272,14 +1260,12 @@
         <v>29</v>
       </c>
       <c r="C15" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="E15" s="8" t="s">
         <v>50</v>
       </c>
+      <c r="E15" s="8"/>
       <c r="F15" s="8"/>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
@@ -1287,11 +1273,19 @@
       <c r="J15" s="8"/>
       <c r="K15" s="8"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="7">
         <v>4</v>
       </c>
-      <c r="D16" s="8"/>
+      <c r="B16" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>51</v>
+      </c>
       <c r="E16" s="8"/>
       <c r="F16" s="8"/>
       <c r="G16" s="8"/>
@@ -1402,21 +1396,22 @@
       </c>
       <c r="C26" t="str" cm="1">
         <f t="array" ref="C26">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Glijvak zonder reststerkte | geen graverij</v>
+        <v>Glijvak zonder reststerkte | geen graverij geen overslag</v>
       </c>
       <c r="D26">
-        <v>3.7</v>
-      </c>
-      <c r="E26" s="25">
-        <v>5E-15</v>
-      </c>
-      <c r="G26" t="str">
-        <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
-        <v/>
-      </c>
-      <c r="H26" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>7.7392563195043733</v>
+        <v>4</v>
+      </c>
+      <c r="E26" s="25"/>
+      <c r="F26">
+        <v>15</v>
+      </c>
+      <c r="G26">
+        <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
+        <v>3.6709661993126968E-51</v>
+      </c>
+      <c r="H26" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -1428,492 +1423,346 @@
       </c>
       <c r="C27" t="str">
         <f t="array" ref="C27">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Glijvak zonder reststerkte | geen graverij</v>
+        <v>Glijvak zonder reststerkte | geen graverij geen overslag</v>
       </c>
       <c r="D27">
-        <v>4.4276</v>
-      </c>
-      <c r="E27" s="25">
-        <v>2E-8</v>
-      </c>
-      <c r="G27" t="str">
-        <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
-        <v/>
-      </c>
-      <c r="H27" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>5.4908517521043487</v>
+        <v>6.4</v>
+      </c>
+      <c r="E27" s="25"/>
+      <c r="F27">
+        <v>4</v>
+      </c>
+      <c r="G27">
+        <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
+        <v>3.1671241833119857E-5</v>
+      </c>
+      <c r="H27" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B28">
         <v>1</v>
       </c>
       <c r="C28" t="str">
         <f t="array" ref="C28">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Glijvak zonder reststerkte | geen graverij</v>
+        <v>Glijvlak zonder reststerkte | geen graverij wel overslag</v>
       </c>
       <c r="D28">
-        <v>5.1651000000000007</v>
-      </c>
-      <c r="E28" s="25">
-        <v>4.0000000000000002E-4</v>
-      </c>
-      <c r="G28" t="str">
-        <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
-        <v/>
-      </c>
-      <c r="H28" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>3.3527947805048282</v>
+        <v>4</v>
+      </c>
+      <c r="E28" s="25"/>
+      <c r="F28">
+        <v>2.5</v>
+      </c>
+      <c r="G28">
+        <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
+        <v>6.2096653257761331E-3</v>
+      </c>
+      <c r="H28" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B29">
         <v>1</v>
       </c>
       <c r="C29" t="str">
         <f t="array" ref="C29">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Glijvak zonder reststerkte | geen graverij</v>
+        <v>Glijvlak zonder reststerkte | graverij geen overslag</v>
       </c>
       <c r="D29">
-        <v>5.9026000000000014</v>
-      </c>
-      <c r="E29" s="25">
-        <v>8.0000000000000004E-4</v>
-      </c>
-      <c r="G29" t="str">
-        <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
-        <v/>
-      </c>
-      <c r="H29" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>3.1559067579218172</v>
+        <v>4</v>
+      </c>
+      <c r="E29" s="25"/>
+      <c r="F29">
+        <v>10</v>
+      </c>
+      <c r="G29">
+        <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
+        <v>7.6198530241604755E-24</v>
+      </c>
+      <c r="H29" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B30">
         <v>1</v>
       </c>
       <c r="C30" t="str">
         <f t="array" ref="C30">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Glijvak zonder reststerkte | geen graverij</v>
+        <v>Glijvlak zonder reststerkte | graverij geen overslag</v>
       </c>
       <c r="D30">
-        <v>6.65</v>
-      </c>
-      <c r="E30" s="25">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="G30" t="str">
-        <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
-        <v/>
-      </c>
-      <c r="H30" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>2.5758293035488999</v>
+        <v>6.4</v>
+      </c>
+      <c r="E30" s="25"/>
+      <c r="F30">
+        <v>3</v>
+      </c>
+      <c r="G30">
+        <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
+        <v>1.3498980316300933E-3</v>
+      </c>
+      <c r="H30" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31">
+        <v>4</v>
+      </c>
+      <c r="B31">
         <v>1</v>
-      </c>
-      <c r="B31">
-        <v>2</v>
       </c>
       <c r="C31" t="str">
         <f t="array" ref="C31">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Overstroming - glijvlak zonder reststerkte | geen graverij</v>
+        <v>Glijvak zonder reststerkte | overslag en graverij</v>
       </c>
       <c r="D31">
-        <v>3</v>
-      </c>
-      <c r="E31">
-        <v>0.5</v>
-      </c>
-      <c r="G31" t="str">
-        <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
-        <v/>
-      </c>
-      <c r="H31" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="F31">
+        <v>7</v>
+      </c>
+      <c r="G31">
+        <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
+        <v>1.2798125438858352E-12</v>
+      </c>
+      <c r="H31" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32">
+        <v>4</v>
+      </c>
+      <c r="B32">
         <v>1</v>
-      </c>
-      <c r="B32">
-        <v>2</v>
       </c>
       <c r="C32" t="str">
         <f t="array" ref="C32">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Overstroming - glijvlak zonder reststerkte | geen graverij</v>
+        <v>Glijvak zonder reststerkte | overslag en graverij</v>
       </c>
       <c r="D32">
-        <v>7</v>
-      </c>
-      <c r="E32">
-        <v>0.99990000000000001</v>
-      </c>
-      <c r="G32" t="str">
-        <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
-        <v/>
-      </c>
-      <c r="H32" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>-3.7190164854557084</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33">
+        <v>6.4</v>
+      </c>
+      <c r="F32">
         <v>2</v>
       </c>
-      <c r="B33">
-        <v>1</v>
-      </c>
+      <c r="G32">
+        <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
+        <v>2.2750131948179191E-2</v>
+      </c>
+      <c r="H32" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C33" t="str">
         <f t="array" ref="C33">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Glijvlak met reststerkte | geen graverij</v>
-      </c>
-      <c r="D33">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="E33" s="25">
-        <v>9.9999999999999995E-7</v>
-      </c>
+        <v/>
+      </c>
+      <c r="E33" s="25"/>
       <c r="G33" t="str">
         <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H33" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>4.7534243088228987</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34">
-        <v>2</v>
-      </c>
-      <c r="B34">
-        <v>1</v>
-      </c>
+      <c r="H33" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C34" t="str">
         <f t="array" ref="C34">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Glijvlak met reststerkte | geen graverij</v>
-      </c>
-      <c r="D34">
-        <v>6.65</v>
-      </c>
-      <c r="E34">
-        <v>0.01</v>
+        <v/>
       </c>
       <c r="G34" t="str">
         <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H34" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>2.3263478740408408</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35">
-        <v>2</v>
-      </c>
-      <c r="B35">
-        <v>2</v>
-      </c>
+      <c r="H34" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C35" t="str">
         <f t="array" ref="C35">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Vervolgmechanismen</v>
-      </c>
-      <c r="D35">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="E35">
-        <v>1E-3</v>
+        <v/>
       </c>
       <c r="G35" t="str">
         <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H35" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>3.0902323061678132</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36">
-        <v>2</v>
-      </c>
-      <c r="B36">
-        <v>2</v>
-      </c>
+      <c r="H35" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C36" t="str">
         <f t="array" ref="C36">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Vervolgmechanismen</v>
-      </c>
-      <c r="D36">
-        <v>6.65</v>
-      </c>
-      <c r="E36">
-        <v>0.5</v>
+        <v/>
       </c>
       <c r="G36" t="str">
         <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H36" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37">
-        <v>2</v>
-      </c>
-      <c r="B37">
-        <v>3</v>
-      </c>
+      <c r="H36" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C37" t="str">
         <f t="array" ref="C37">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Overstroming - glijvlak/vervolgmechanismen | geen graverij</v>
-      </c>
-      <c r="D37">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="E37">
-        <v>1E-4</v>
+        <v/>
       </c>
       <c r="G37" t="str">
         <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H37" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>3.71901648545568</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38">
-        <v>2</v>
-      </c>
-      <c r="B38">
-        <v>3</v>
-      </c>
+      <c r="H37" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C38" t="str">
         <f t="array" ref="C38">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Overstroming - glijvlak/vervolgmechanismen | geen graverij</v>
-      </c>
-      <c r="D38">
-        <v>6.65</v>
-      </c>
-      <c r="E38">
-        <v>0.99990000000000001</v>
+        <v/>
       </c>
       <c r="G38" t="str">
         <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H38" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>-3.7190164854557084</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39">
-        <v>3</v>
-      </c>
-      <c r="B39">
-        <v>1</v>
-      </c>
+      <c r="H38" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C39" t="str">
         <f t="array" ref="C39">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Glijvlak zonder reststerkte | graverij</v>
-      </c>
-      <c r="D39">
-        <v>3.7</v>
-      </c>
-      <c r="E39" s="25">
-        <v>4.9999999999999997E-12</v>
-      </c>
+        <v/>
+      </c>
+      <c r="E39" s="25"/>
       <c r="G39" t="str">
         <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H39" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>6.806502490740626</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40">
-        <v>3</v>
-      </c>
-      <c r="B40">
-        <v>1</v>
-      </c>
+      <c r="H39" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C40" t="str">
         <f t="array" ref="C40">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Glijvlak zonder reststerkte | graverij</v>
-      </c>
-      <c r="D40">
-        <v>4.4276</v>
-      </c>
-      <c r="E40" s="25">
-        <v>1.9999999999999999E-6</v>
-      </c>
+        <v/>
+      </c>
+      <c r="E40" s="25"/>
       <c r="G40" t="str">
         <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H40" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>4.6113823623026677</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41">
-        <v>3</v>
-      </c>
-      <c r="B41">
-        <v>1</v>
-      </c>
+      <c r="H40" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C41" t="str">
         <f t="array" ref="C41">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Glijvlak zonder reststerkte | graverij</v>
-      </c>
-      <c r="D41">
-        <v>5.1651000000000007</v>
-      </c>
-      <c r="E41" s="25">
-        <v>4.0000000000000001E-3</v>
-      </c>
+        <v/>
+      </c>
+      <c r="E41" s="25"/>
       <c r="G41" t="str">
         <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H41" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>2.6520698079021954</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42">
-        <v>3</v>
-      </c>
-      <c r="B42">
-        <v>1</v>
-      </c>
+      <c r="H41" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C42" t="str">
         <f t="array" ref="C42">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Glijvlak zonder reststerkte | graverij</v>
-      </c>
-      <c r="D42">
-        <v>5.9026000000000014</v>
-      </c>
-      <c r="E42" s="25">
-        <v>8.0000000000000002E-3</v>
-      </c>
+        <v/>
+      </c>
+      <c r="E42" s="25"/>
       <c r="G42" t="str">
         <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H42" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>2.4089155458154612</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43">
-        <v>3</v>
-      </c>
-      <c r="B43">
-        <v>1</v>
-      </c>
+      <c r="H42" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C43" t="str">
         <f t="array" ref="C43">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Glijvlak zonder reststerkte | graverij</v>
-      </c>
-      <c r="D43">
-        <v>6.65</v>
-      </c>
-      <c r="E43" s="25">
-        <v>0.05</v>
-      </c>
+        <v/>
+      </c>
+      <c r="E43" s="25"/>
       <c r="G43" t="str">
         <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H43" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>1.6448536269514726</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44">
-        <v>3</v>
-      </c>
-      <c r="B44">
-        <v>2</v>
-      </c>
+      <c r="H43" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C44" t="str">
         <f t="array" ref="C44">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Overstroming - glijvlak zonder reststerkte | graverij</v>
-      </c>
-      <c r="D44">
-        <v>3</v>
-      </c>
-      <c r="E44">
-        <v>0.5</v>
+        <v/>
       </c>
       <c r="G44" t="str">
         <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H44" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A45">
-        <v>3</v>
-      </c>
-      <c r="B45">
-        <v>2</v>
-      </c>
+      <c r="H44" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C45" t="str">
         <f t="array" ref="C45">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
-        <v>Overstroming - glijvlak zonder reststerkte | graverij</v>
-      </c>
-      <c r="D45">
-        <v>7</v>
-      </c>
-      <c r="E45">
-        <v>0.99990000000000001</v>
+        <v/>
       </c>
       <c r="G45" t="str">
         <f>IF(FCPunten5[[#This Row],[Beta_h]]="","",_xlfn.NORM.S.DIST(-1*FCPunten5[[#This Row],[Beta_h]],TRUE))</f>
         <v/>
       </c>
-      <c r="H45" s="13">
-        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
-        <v>-3.7190164854557084</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H45" s="13" t="str">
+        <f>IF(FCPunten5[[#This Row],[Pf_h]]="", "",-_xlfn.NORM.S.INV(FCPunten5[[#This Row],[Pf_h]]))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C46" t="str">
         <f t="array" ref="C46">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
         <v/>
@@ -1927,7 +1776,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C47" t="str">
         <f t="array" ref="C47">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
         <v/>
@@ -1941,7 +1790,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C48" t="str">
         <f t="array" ref="C48">IF(SUM(FCPunten5[[#This Row],[Faalpad_ID]:[Knoop_ID]])&gt;=2,INDEX(FaalpadenGegevenScenario4[[Initiele_gebeurtenis]:[Vervolggebeurtenis_7]],FCPunten5[[#This Row],[Faalpad_ID]],FCPunten5[[#This Row],[Knoop_ID]]),"")</f>
         <v/>
@@ -2139,7 +1988,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -2152,31 +2001,91 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="B2" s="10">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="9"/>
-      <c r="B3" s="10"/>
+      <c r="A3" s="9">
+        <v>2.1</v>
+      </c>
+      <c r="B3" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="9"/>
-      <c r="B4" s="10"/>
+      <c r="A4" s="9">
+        <v>3</v>
+      </c>
+      <c r="B4" s="14">
+        <v>1E-10</v>
+      </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="9"/>
-      <c r="B5" s="10"/>
+      <c r="A5" s="9">
+        <v>3.5</v>
+      </c>
+      <c r="B5" s="14">
+        <v>1E-4</v>
+      </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="9"/>
-      <c r="B6" s="10"/>
+      <c r="A6" s="9">
+        <v>4.5</v>
+      </c>
+      <c r="B6" s="14">
+        <v>1E-3</v>
+      </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="11"/>
-      <c r="B7" s="12"/>
+      <c r="A7" s="9">
+        <v>5.5</v>
+      </c>
+      <c r="B7" s="14">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="9">
+        <v>5.95</v>
+      </c>
+      <c r="B8" s="14">
+        <v>6.4607700000000004E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="9">
+        <v>6</v>
+      </c>
+      <c r="B9" s="14">
+        <v>0.39505699999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="9">
+        <v>6.05</v>
+      </c>
+      <c r="B10" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="9">
+        <v>6.1</v>
+      </c>
+      <c r="B11" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="9">
+        <v>6.15</v>
+      </c>
+      <c r="B12" s="14">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>